<commit_message>
Add personalized kindergarten recommendation
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R6254ba9883ae44fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R50f6f97b775c44e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Ra1cf1594e9b14def"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="Rdefb00047cb74d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R62a1d3664c26424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rc35ffce7be104722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R42b7c8c70d074d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Ra8e39f07cc504b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R149a1f881fff4665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R96ccad1547524a67"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Restructure page as decision report
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rc35ffce7be104722"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R42b7c8c70d074d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Ra8e39f07cc504b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R149a1f881fff4665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R96ccad1547524a67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rc679f67b560e4ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rb2d627211118405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R4063fa3306954475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R05e3b438968246d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R7533fcaaffe34f81"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add detailed recommendations and enrollment todos
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rc679f67b560e4ffa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rb2d627211118405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R4063fa3306954475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R05e3b438968246d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R7533fcaaffe34f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R5a2e3f56cee145ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R58e5f50aa2454e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Rc2496c2bf8cc49a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R54b2e9fcfad945f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="Re8dbaa1ba799499c"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add private kindergarten fallback recommendations
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R5a2e3f56cee145ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R58e5f50aa2454e62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Rc2496c2bf8cc49a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R54b2e9fcfad945f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="Re8dbaa1ba799499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rf7670484217e432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rd20e8f95313042f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R420068a996c9489c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="Rf10aa64b72534c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R2a1d920d79294623"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Polish Amap-based decision report
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R0327cee29f8c41f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rb502e0a547f24228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R668be1861abf42ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R105f884346764fa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R17a3f3a0e49c4d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R7287790bb28248c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R3da8c0f6ebbb4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R9fa1440029174752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="Rfb603b6bf225419c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R5c45b33935aa4b0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -295,7 +295,7 @@
         <x:v>高德增强字段</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>已接入</x:v>
+        <x:v>101/127</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
         <x:v>已批量补POI名称、经纬度和到网易上海西岸研发中心的高德直线距离；低置信匹配保留为待核验。</x:v>

</xml_diff>

<commit_message>
Improve kindergarten decision report
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R7287790bb28248c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R3da8c0f6ebbb4ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="R9fa1440029174752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="Rfb603b6bf225419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R5c45b33935aa4b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rfb7f32c519f44300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rc1d19fd76cf44df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Rc2be6762bca146c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R96fe5e3c6ee44778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="Rfc2794de94224cc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10404,65 +10404,129 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
-        <x:v>公办园部地址主来源</x:v>
+        <x:v>2026招生工作方案</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>上海本地宝《上海市徐汇区公办幼儿园名单一览》，内容来源标注为上海学前教育网，2024-03-25：https://m.sh.bendibao.com/edu/284155.html</x:v>
+        <x:v>https://sh.bendibao.com/news/2026415/305294.shtm；用于判断户籍优先、外省市户籍排序、录取批次、报名验证和统筹规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>民办/私立地址与电话来源</x:v>
+        <x:v>2026报名材料</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>上海本地宝《上海市徐汇区民办幼儿园名单一览》，内容来源标注为上海学前教育网，2024-03-25：https://sh.bendibao.com/edu/2024325/284155_2.shtm</x:v>
+        <x:v>https://m.sh.bendibao.com/edu/305384.html；用于核对非沪籍幼儿、父母居住证、租赁合同、居住登记和地址一致性要求。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
-        <x:v>高德MCP接入口径</x:v>
+        <x:v>上海居住证办理条件</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>目标办公点：西岸网易研发中心；高德匹配为“网易上海西岸研发中心”。用关键词搜索和距离测量补齐高德POI、经纬度和距离。</x:v>
+        <x:v>https://m.sh.bendibao.com/zffw/285087.html；用于确认居住登记、合法稳定住所、租赁合同/备案等材料链要求。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
-        <x:v>高德检索口径</x:v>
+        <x:v>公办园部地址主来源</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>表格中的高德链接使用“上海市徐汇区 + 幼儿园名 + 园区名 + 地址”生成，用于逐点打开核验。</x:v>
+        <x:v>上海本地宝《上海市徐汇区公办幼儿园名单一览》，内容来源标注为上海学前教育网，2024-03-25：https://m.sh.bendibao.com/edu/284155.html</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
-        <x:v>A级</x:v>
+        <x:v>民办/私立地址与电话来源</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>园部地址在公办园地址清单中明确列出，且无明显冲突。</x:v>
+        <x:v>上海本地宝《上海市徐汇区民办幼儿园名单一览》，内容来源标注为上海学前教育网，2024-03-25：https://sh.bendibao.com/edu/2024325/284155_2.shtm</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
-        <x:v>B级</x:v>
+        <x:v>高德MCP接入口径</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>公开资料有变更、合并或地址冲突，位置大体可定位，但实际入读园区需电话确认。</x:v>
+        <x:v>目标办公点：西岸网易研发中心；高德匹配为“网易上海西岸研发中心”。用关键词搜索和距离测量补齐高德POI、经纬度和距离。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="str">
-        <x:v>C级</x:v>
+        <x:v>高德增强落地数据</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>仅有第三方或地图信息，缺少官方交叉验证。本表目前未使用C级作为主确认。</x:v>
+        <x:v>data/amap_enrichment.json；用于补充POI名称、POI地址、经纬度、距公司直线距离。低置信匹配不写入推荐结论。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="3" t="str">
+        <x:v>高德检索口径</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>表格中的高德链接使用“上海市徐汇区 + 幼儿园名 + 园区名 + 地址”生成，用于逐点打开核验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="3" t="str">
+        <x:v>贝壳租房参数</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>data/beike_rental_filter_schema.json；用于生成徐汇及二级商圈结构化租房链接，固定token：rt200600000001brp0erp10000l2l3ra4ra5ie1。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="3" t="str">
+        <x:v>贝壳租房口径</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>https://sh.zu.ke.com/；房源价格和库存实时变化，本页只保存查询条件和入口，不固化具体房源。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="3" t="str">
+        <x:v>办公点参考</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>https://www.chooffice.com/1357.html；用于确认西岸网易研发中心靠近龙耀路、徐汇滨江一带。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="3" t="str">
+        <x:v>第三方园所资料</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>上哪学、021school、园所公开页面等；用于交叉核对部分民办园电话、收费、托幼一体和地址差异，最终以园所电话确认为准。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="3" t="str">
+        <x:v>A级</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="str">
+        <x:v>园部地址在公办园地址清单中明确列出，且无明显冲突。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="3" t="str">
+        <x:v>B级</x:v>
+      </x:c>
+      <x:c r="B17" s="3" t="str">
+        <x:v>公开资料有变更、合并或地址冲突，位置大体可定位，但实际入读园区需电话确认。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="3" t="str">
+        <x:v>C级</x:v>
+      </x:c>
+      <x:c r="B18" s="3" t="str">
+        <x:v>仅有第三方或地图信息，缺少官方交叉验证。本表目前未使用C级作为主确认。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="3" t="str">
         <x:v>电话确认重点</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="str">
+      <x:c r="B19" s="3" t="str">
         <x:v>汇星幼儿园北园；复旦大学附属徐汇实验幼儿园；区域内自主招生、扩招园、民办/私立园。</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add dial links to kindergarten phones
</commit_message>
<xml_diff>
--- a/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
+++ b/outputs/徐汇区幼儿园园区位置与择园参考.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="Rfb7f32c519f44300"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="Rc1d19fd76cf44df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Rc2be6762bca146c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="R96fe5e3c6ee44778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="Rfc2794de94224cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="1" r:id="R7cc67c46c7f24172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="招生主体" sheetId="2" r:id="R3953e62910ab425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="园区点位" sheetId="3" r:id="Rc6167b0f7de54ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="片区统计" sheetId="4" r:id="Rc45ae9785eca477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与核验规则" sheetId="5" r:id="R4d1ebac9885c4e9f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>